<commit_message>
finalização da aba geral
</commit_message>
<xml_diff>
--- a/relationships_level_results.xlsx
+++ b/relationships_level_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,15 +461,20 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Auto_created</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>DAX_uses</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>From_column</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>To_column</t>
         </is>
@@ -478,12 +483,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>'Vendas'[ID_Cliente] N &lt;- 1 'Clientes'[ID_Cliente]</t>
+          <t>'d_calendario'[DataId] N &lt;- 1 'LocalDateTable_b29d074d-15a8-4404-91ac-86d4831a03e8'[Date]</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AutoDetected_ae59214a-34ea-4ed2-beab-5beb64070c47</t>
+          <t>27dcdd83-cfda-41eb-9ef5-fa028875b3fe</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -508,29 +513,34 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Vendas[ID_Cliente]</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Clientes[ID_Cliente]</t>
+          <t>d_calendario[DataId]</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>LocalDateTable_b29d074d-15a8-4404-91ac-86d4831a03e8[Date]</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>'Vendas'[ID_Produto] N &lt;- 1 'Produtos'[ID_Produto]</t>
+          <t>'f_vendas'[d_produtos.Nome_Produto] N &lt;- 1 'produtosOutros'[d_produtos.Nome_Produto]</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AutoDetected_92e57305-38ae-4bce-957b-2616ff73bd3e</t>
+          <t>782be332-6460-204e-8b10-5ef6150686a8</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -555,64 +565,230 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Vendas[ID_Produto]</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Produtos[ID_Produto]</t>
+          <t>f_vendas[d_produtos.Nome_Produto]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>produtosOutros[d_produtos.Nome_Produto]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>'Vendas'[ID_Vendedor] N &lt;- 1 'Vendedores'[ID_Vendedor]</t>
+          <t>'f_vendas'[Data] N &lt;- 1 'd_calendario'[DataId]</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>b368c512-6b31-5785-f80b-3a7dcd3f10e3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> N &lt;- 1 </t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Used</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>f_vendas[Data]</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>d_calendario[DataId]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>'f_vendas'[ID_Cliente] N &lt;- 1 'd_clientes'[ID_Cliente]</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AutoDetected_ae59214a-34ea-4ed2-beab-5beb64070c47</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> N &lt;- 1 </t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Used</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>f_vendas[ID_Cliente]</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>d_clientes[ID_Cliente]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>'f_vendas'[ID_Produto] N &lt;- 1 'd_produtos'[ID_Produto]</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AutoDetected_92e57305-38ae-4bce-957b-2616ff73bd3e</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> N &lt;- 1 </t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Used</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>f_vendas[ID_Produto]</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>d_produtos[ID_Produto]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>'f_vendas'[ID_Vendedor] N &lt;- 1 'd_vendedores'[ID_Vendedor]</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>AutoDetected_c43d17d1-7fe5-430f-bc1f-746bb8b7c175</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t xml:space="preserve"> N &lt;- 1 </t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Used</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Vendas[ID_Vendedor]</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Vendedores[ID_Vendedor]</t>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>f_vendas[ID_Vendedor]</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>d_vendedores[ID_Vendedor]</t>
         </is>
       </c>
     </row>

</xml_diff>